<commit_message>
feat: HypoLedger integration — architecture v5, Excel-Sync-Protocol, README, memory
- architecture-v5-2026-04-22.md: Master Data Log 10→11 sheets; daily-trade-rec §5 adds HypoLedger append (Step 8.5); signal-review §5 adds HypoLedger read + mark-to-market + dim-14; Mermaid Excel node updated
- framework/architecture/README.md: v5 entry added
- framework/Excel-Sync-Protocol.md: stale hypo-ledger-2026.md row updated to HypoLedger dedicated sheet; header date updated to 2026-04-22
- master-data-log.xlsx README sheet: HypoLedger block inserted (rows 39-42); stale SignalLedger description fixed

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Trade/master-data-log.xlsx
+++ b/Trade/master-data-log.xlsx
@@ -40,7 +40,7 @@
     <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="168" formatCode="0.00%;(0.00%);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -129,6 +129,9 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="10">
@@ -228,7 +231,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -290,6 +293,7 @@
     <xf numFmtId="168" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -18970,7 +18974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B63"/>
+  <dimension ref="A1:B67"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.25"/>
   <cols>
     <col width="25" customWidth="1" style="15" min="1" max="1"/>
@@ -19053,7 +19057,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>All promoted and near-miss signals. Mirrors hypo-ledger-2026.md in structured form.</t>
+          <t>All promoted and near-miss signals. Append-only ledger — one row per signal.</t>
         </is>
       </c>
     </row>
@@ -19260,163 +19264,196 @@
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="15">
-      <c r="A39" s="6" t="n"/>
+      <c r="A39" s="33" t="inlineStr">
+        <is>
+          <t>HypoLedger</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>All formally promoted signals (Sum&gt;=3, checklist PASS) tracked at recommendation price for system efficacy measurement.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="15">
-      <c r="A40" s="10" t="inlineStr">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Producer: daily-trade-rec skill Step 8.5 (appends H### rows at rec time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="15" customHeight="1" s="15">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Consumer: signal-review (marks to market weekly, produces dim-14 efficacy report in PerformanceStats)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="15" customHeight="1" s="15">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Key columns: H_ID, Rec_Date, Asset, Direction, Entry_Price_Rec, Stop_Rec, TP1_Rec, Hypo_Entry_Price, Hypo_Current_Price, Hypo_PnL_%, Actual_Taken, Actual_PnL_%</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="15" customHeight="1" s="15">
+      <c r="A43" s="6" t="n"/>
+    </row>
+    <row r="44" ht="15" customHeight="1" s="15">
+      <c r="A44" s="10" t="inlineStr">
         <is>
           <t>RULES:</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="15" customHeight="1" s="15">
-      <c r="A41" s="11" t="inlineStr">
-        <is>
-          <t>1. SignalLedger is append-only. Never delete or retroactively edit rows.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="15" customHeight="1" s="15">
-      <c r="A42" s="11" t="inlineStr">
-        <is>
-          <t>2. DailyVariables: one row per trading day. Overwrite only if same-day correction (note in Source_Brief).</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="15" customHeight="1" s="15">
-      <c r="A43" s="11" t="inlineStr">
-        <is>
-          <t>3. VariableRegistry: variables can change status but are never deleted. Rejected/Retired variables stay for audit trail.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="15" customHeight="1" s="15">
-      <c r="A44" s="11" t="inlineStr">
-        <is>
-          <t>4. Markdown files remain the human-readable presentation layer. This workbook is the analytical layer.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="15">
       <c r="A45" s="11" t="inlineStr">
         <is>
-          <t>5. If markdown and Excel diverge, Excel is source of truth for quantitative data.</t>
+          <t>1. SignalLedger is append-only. Never delete or retroactively edit rows.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="15">
-      <c r="A46" s="6" t="n"/>
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>2. DailyVariables: one row per trading day. Overwrite only if same-day correction (note in Source_Brief).</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="15">
-      <c r="A47" s="10" t="inlineStr">
-        <is>
-          <t>VARIABLE DISCOVERY SYSTEM:</t>
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t>3. VariableRegistry: variables can change status but are never deleted. Rejected/Retired variables stay for audit trail.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="15">
       <c r="A48" s="11" t="inlineStr">
         <is>
+          <t>4. Markdown files remain the human-readable presentation layer. This workbook is the analytical layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="15" customHeight="1" s="15">
+      <c r="A49" s="11" t="inlineStr">
+        <is>
+          <t>5. If markdown and Excel diverge, Excel is source of truth for quantitative data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="15" customHeight="1" s="15">
+      <c r="A50" s="6" t="n"/>
+    </row>
+    <row r="51" ht="15" customHeight="1" s="15">
+      <c r="A51" s="10" t="inlineStr">
+        <is>
+          <t>VARIABLE DISCOVERY SYSTEM:</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="15" customHeight="1" s="15">
+      <c r="A52" s="11" t="inlineStr">
+        <is>
           <t>Status Ladder:</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="15" customHeight="1" s="15">
-      <c r="A49" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Candidate — plausible idea, not yet assessed</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="15" customHeight="1" s="15">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Watchlist — weak or mixed evidence, worth tracking over time</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="15" customHeight="1" s="15">
-      <c r="A51" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Under Review — being actively assessed with data</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="15" customHeight="1" s="15">
-      <c r="A52" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Provisionally Useful — seems helpful but not fully trusted (pilot phase)</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="15">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Approved — good enough for regular use, pending Grade A evidence</t>
+          <t xml:space="preserve">  Candidate — plausible idea, not yet assessed</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="15">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Grade A — strong evidence, repeated usefulness, in core methodology</t>
+          <t xml:space="preserve">  Watchlist — weak or mixed evidence, worth tracking over time</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="15">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Rejected — failed screening or proved unhelpful; kept for audit trail</t>
+          <t xml:space="preserve">  Under Review — being actively assessed with data</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="15">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Retired — was useful but no longer (regime change, decay, etc.)</t>
+          <t xml:space="preserve">  Provisionally Useful — seems helpful but not fully trusted (pilot phase)</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="15">
-      <c r="A57" s="6" t="n"/>
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Approved — good enough for regular use, pending Grade A evidence</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="15">
-      <c r="A58" s="11" t="inlineStr">
-        <is>
-          <t>Review Cadence:</t>
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Grade A — strong evidence, repeated usefulness, in core methodology</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="15">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Daily: literature-review and market-brief can add Candidate entries</t>
+          <t xml:space="preserve">  Rejected — failed screening or proved unhelpful; kept for audit trail</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="15">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Weekly: signal-review flags blocking patterns that suggest variable gaps</t>
+          <t xml:space="preserve">  Retired — was useful but no longer (regime change, decay, etc.)</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="15">
-      <c r="A61" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Monthly: bootstrap-review and quarterly-review assess Watchlist promotions</t>
-        </is>
-      </c>
+      <c r="A61" s="6" t="n"/>
     </row>
     <row r="62" ht="15" customHeight="1" s="15">
-      <c r="A62" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Quarterly: formal promote/demote/reject decisions with Gerald sign-off</t>
+      <c r="A62" s="11" t="inlineStr">
+        <is>
+          <t>Review Cadence:</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="15">
       <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Daily: literature-review and market-brief can add Candidate entries</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Weekly: signal-review flags blocking patterns that suggest variable gaps</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Monthly: bootstrap-review and quarterly-review assess Watchlist promotions</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Quarterly: formal promote/demote/reject decisions with Gerald sign-off</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Semi-annual: literature-review deep scan for new academic variables</t>
         </is>

</xml_diff>

<commit_message>
routine: hypo-ledger mark-to-market 2026-04-22
H001 EWY +2.80% | H003 INTC +8.06% (earnings tonight) | H004 Gold -0.93%
H005 QQQ FLAGGED +1.47% | H006 SPY -0.56% | H007 EWJ -1.17%
H008/H009/H010 PENDING — INTC/AAPL/GOOGL earnings gate Apr-23
Hypo wtd avg PnL (OPEN): ~+2.0%

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Trade/master-data-log.xlsx
+++ b/Trade/master-data-log.xlsx
@@ -2384,7 +2384,7 @@
         <v>146</v>
       </c>
       <c r="S2" s="21" t="n">
-        <v>152.33</v>
+        <v>150.09</v>
       </c>
       <c r="T2" s="24">
         <f>(S2-R2)/R2</f>
@@ -2551,7 +2551,7 @@
         <v>62</v>
       </c>
       <c r="S4" s="21" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="T4" s="24">
         <f>(S4-R4)/R4</f>
@@ -2647,7 +2647,7 @@
         <v>4830</v>
       </c>
       <c r="S5" s="21" t="n">
-        <v>4808</v>
+        <v>4785.16</v>
       </c>
       <c r="T5" s="24">
         <f>(S5-R5)/R5</f>
@@ -2835,7 +2835,7 @@
         <v>710.14</v>
       </c>
       <c r="S7" s="21" t="n">
-        <v>706</v>
+        <v>706.14</v>
       </c>
       <c r="T7" s="24">
         <f>(S7-R7)/R7</f>
@@ -3198,6 +3198,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="29" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: HypoLedger backfill complete — H011/H012 FLAGGED + Apr-22 MTM
Backlog complete from earliest available trade rec (2026-04-14):
- Apr-14: no promotions (EWY fail-loud on missing Grade A R-overlay) — confirmed
- Apr-15: H001 EWY OPEN, H002 TSM VOIDED, H003 INTC OPEN — confirmed
- Apr-16: H004 Gold OPEN, H005 QQQ FLAGGED — confirmed
  + H011 GOOGL FLAGGED (NEW: residual +30.52% T unblocked; blocked by correlation gate + post-rally)
  + H012 SPY FLAGGED (NEW: Sum+3 blocked by QQQ correlation; promoted 4 days later as H006)
- Apr-17: no new promotions (all existing open or correlation-blocked) — confirmed
- Apr-20: H006 SPY OPEN — confirmed
- Apr-21: H007 EWJ OPEN, H008/H009/H010 PENDING — confirmed

Apr-22 mark-to-market: H011 GOOGL +0.09%, H012 SPY +0.89%
COUNTIF/AVERAGEIF formulas extended to rows 2:13

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Trade/master-data-log.xlsx
+++ b/Trade/master-data-log.xlsx
@@ -134,7 +134,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -189,6 +189,12 @@
         <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -231,7 +237,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -294,6 +300,8 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2157,7 +2165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y21"/>
+  <dimension ref="A1:Y22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="15" min="1" max="1"/>
@@ -3198,106 +3206,278 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
+    <row r="12">
+      <c r="A12" s="34" t="inlineStr">
+        <is>
+          <t>H011</t>
+        </is>
+      </c>
+      <c r="B12" s="35" t="n">
+        <v>46128</v>
+      </c>
+      <c r="C12" s="34" t="inlineStr">
+        <is>
+          <t>trade-rec-2026-04-16 v3</t>
+        </is>
+      </c>
+      <c r="D12" s="34" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="E12" s="34" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="F12" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="K12" s="34" t="n">
+        <v>337.12</v>
+      </c>
+      <c r="L12" s="34" t="n">
+        <v>297</v>
+      </c>
+      <c r="M12" s="34" t="n">
+        <v>360</v>
+      </c>
+      <c r="N12" s="34" t="n">
+        <v>380</v>
+      </c>
+      <c r="O12" s="34" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="P12" s="34" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="Q12" s="34" t="inlineStr">
+        <is>
+          <t>FLAGGED</t>
+        </is>
+      </c>
+      <c r="R12" s="34" t="n">
+        <v>337.12</v>
+      </c>
+      <c r="S12" s="34" t="n">
+        <v>337.42</v>
+      </c>
+      <c r="T12" s="34">
+        <f>(S12-R12)/R12</f>
+        <v/>
+      </c>
+      <c r="U12" s="34" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="V12" s="34" t="n"/>
+      <c r="W12" s="34" t="n"/>
+      <c r="X12" s="34" t="n"/>
+      <c r="Y12" s="34" t="inlineStr">
+        <is>
+          <t>Flagged Sum+3 Apr-16 (residual +30.52%, T unblocked). Not promoted: correlation gate (EWY+INTC+GOOGL equity heat ~13.75%) + post-rally entry risk (+6.01% same day) + FOMC Apr-28 timing. Earnings Apr-22 now past. H010 = Apr-21 PENDING re-entry (post-earnings contingent).</t>
+        </is>
+      </c>
+    </row>
     <row r="13">
-      <c r="A13" s="29" t="inlineStr">
+      <c r="A13" s="34" t="inlineStr">
+        <is>
+          <t>H012</t>
+        </is>
+      </c>
+      <c r="B13" s="35" t="n">
+        <v>46128</v>
+      </c>
+      <c r="C13" s="34" t="inlineStr">
+        <is>
+          <t>trade-rec-2026-04-16 v3</t>
+        </is>
+      </c>
+      <c r="D13" s="34" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E13" s="34" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="F13" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="K13" s="34" t="n">
+        <v>699.9400000000001</v>
+      </c>
+      <c r="L13" s="34" t="n">
+        <v>685</v>
+      </c>
+      <c r="M13" s="34" t="n">
+        <v>720</v>
+      </c>
+      <c r="N13" s="34" t="n">
+        <v>740</v>
+      </c>
+      <c r="O13" s="34" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="P13" s="34" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="Q13" s="34" t="inlineStr">
+        <is>
+          <t>FLAGGED</t>
+        </is>
+      </c>
+      <c r="R13" s="34" t="n">
+        <v>699.9400000000001</v>
+      </c>
+      <c r="S13" s="34" t="n">
+        <v>706.14</v>
+      </c>
+      <c r="T13" s="34">
+        <f>(S13-R13)/R13</f>
+        <v/>
+      </c>
+      <c r="U13" s="34" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="V13" s="34" t="n"/>
+      <c r="W13" s="34" t="n"/>
+      <c r="X13" s="34" t="n"/>
+      <c r="Y13" s="34" t="inlineStr">
+        <is>
+          <t>Flagged Sum+3 Apr-16. Not promoted: dominated by open QQQ position (same broad equity risk-on regime variable). Apr-17 rec explicitly blocks via correlation gate (Risk Rules §5 item 3). Formally promoted 4 days later at $710.14 (H006 Apr-20). Counterfactual: Apr-16 FLAGGED entry $699.94 vs Apr-20 formal entry $710.14 = $10.20/share better entry. Hypo +0.89% vs H006 hypo -0.56% as of Apr-22.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>PERFORMANCE SUMMARY (auto-updated by signal-review)</t>
         </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="30" t="inlineStr">
-        <is>
-          <t>Formally Promoted (OPEN+PENDING+FLAGGED)</t>
-        </is>
-      </c>
-      <c r="B14" s="31">
-        <f>COUNTIF(Q2:Q11,"OPEN")+COUNTIF(Q2:Q11,"PENDING")+COUNTIF(Q2:Q11,"FLAGGED")</f>
-        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="30" t="inlineStr">
         <is>
-          <t>OPEN (marked-to-market)</t>
+          <t>Formally Promoted (OPEN+PENDING+FLAGGED)</t>
         </is>
       </c>
       <c r="B15" s="31">
-        <f>COUNTIF(Q2:Q11,"OPEN")</f>
+        <f>COUNTIF(Q2:Q13,"OPEN")+COUNTIF(Q2:Q13,"PENDING")+COUNTIF(Q2:Q13,"FLAGGED")</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>PENDING (entry trigger)</t>
+          <t>OPEN (marked-to-market)</t>
         </is>
       </c>
       <c r="B16" s="31">
-        <f>COUNTIF(Q2:Q11,"PENDING")</f>
+        <f>COUNTIF(Q2:Q13,"OPEN")</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="30" t="inlineStr">
         <is>
-          <t>VOIDED (de-promoted same session)</t>
+          <t>PENDING (entry trigger)</t>
         </is>
       </c>
       <c r="B17" s="31">
-        <f>COUNTIF(Q2:Q11,"VOIDED")</f>
+        <f>COUNTIF(Q2:Q13,"PENDING")</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="30" t="inlineStr">
         <is>
-          <t>FLAGGED (Sum&gt;=3, not formally promoted)</t>
+          <t>VOIDED (de-promoted same session)</t>
         </is>
       </c>
       <c r="B18" s="31">
-        <f>COUNTIF(Q2:Q11,"FLAGGED")</f>
+        <f>COUNTIF(Q2:Q13,"VOIDED")</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="30" t="inlineStr">
         <is>
-          <t>Hypo Avg PnL% -- OPEN signals</t>
-        </is>
-      </c>
-      <c r="B19" s="32">
-        <f>AVERAGEIF(Q2:Q11,"OPEN",T2:T11)</f>
+          <t>FLAGGED (Sum&gt;=3, not formally promoted)</t>
+        </is>
+      </c>
+      <c r="B19" s="31">
+        <f>COUNTIF(Q2:Q13,"FLAGGED")</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="30" t="inlineStr">
         <is>
-          <t>Actual Avg PnL% -- closed YES</t>
+          <t>Hypo Avg PnL% -- OPEN signals</t>
         </is>
       </c>
       <c r="B20" s="32">
-        <f>AVERAGEIFS(X2:X11,U2:U11,"YES",W2:W11,"&lt;&gt;"&amp;"")</f>
+        <f>AVERAGEIF(Q2:Q13,"OPEN",T2:T13)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="30" t="inlineStr">
         <is>
+          <t>Actual Avg PnL% -- closed YES</t>
+        </is>
+      </c>
+      <c r="B21" s="32">
+        <f>AVERAGEIFS(X2:X13,U2:U13,"YES",W2:W13,"&lt;&gt;"&amp;"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="30" t="inlineStr">
+        <is>
           <t>Last updated</t>
         </is>
       </c>
-      <c r="B21" s="31">
+      <c r="B22" s="31">
         <f>TEXT(NOW(),"YYYY-MM-DD HH:MM UTC+8")</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A13:H13"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>